<commit_message>
Add separate exam search tabs
</commit_message>
<xml_diff>
--- a/2026-2027-guz-vize.xlsx
+++ b/2026-2027-guz-vize.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30619"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\l\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C493007A-BD1B-4BD6-B5C0-027BD5AFD758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DBE5897D-9225-433D-99AC-53F443FA5E65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4056" uniqueCount="581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4056" uniqueCount="580">
   <si>
     <t>Ders Kodu</t>
   </si>
@@ -1161,6 +1161,9 @@
     <t>Dr. Öğr. Üyesi Gökçe Özkılıççı</t>
   </si>
   <si>
+    <t>Prof. Dr. Seda BAĞDATLI KALKAN</t>
+  </si>
+  <si>
     <t>PSİ355</t>
   </si>
   <si>
@@ -1470,6 +1473,9 @@
     <t>YBS107</t>
   </si>
   <si>
+    <t>Dr. Öğr. Üyesi Gökçe ÖZKILIÇCI</t>
+  </si>
+  <si>
     <t>YBS201</t>
   </si>
   <si>
@@ -1512,15 +1518,9 @@
     <t>BA301</t>
   </si>
   <si>
-    <t>Dr. Öğr. Üyesi Gökçe ÖZKILIÇCI</t>
-  </si>
-  <si>
     <t>F-104</t>
   </si>
   <si>
-    <t>Prof. Dr. Seda BAĞDATLI KALKAN</t>
-  </si>
-  <si>
     <t>Dr. Öğr. Üyesi Onur YAMANER</t>
   </si>
   <si>
@@ -1552,9 +1552,6 @@
   </si>
   <si>
     <t>Dr. Öğr. Üyesi Engincan Yıldız</t>
-  </si>
-  <si>
-    <t>Büşra Bur Doğan</t>
   </si>
   <si>
     <t>İŞL576</t>
@@ -1963,7 +1960,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="22">
+  <fills count="23">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2087,6 +2084,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2475,7 +2478,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="170">
+  <cellXfs count="166">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2781,27 +2784,23 @@
     <xf numFmtId="0" fontId="19" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -17012,13 +17011,13 @@
       <c r="G400" s="135">
         <v>0.67708333333333337</v>
       </c>
-      <c r="H400" s="162" t="s">
+      <c r="H400" s="136" t="s">
         <v>229</v>
       </c>
-      <c r="I400" s="162" t="s">
+      <c r="I400" s="136" t="s">
         <v>234</v>
       </c>
-      <c r="J400" s="163"/>
+      <c r="J400" s="133"/>
     </row>
     <row r="401" spans="1:10">
       <c r="A401" s="133" t="s">
@@ -17042,13 +17041,13 @@
       <c r="G401" s="135">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H401" s="163" t="s">
+      <c r="H401" s="133" t="s">
         <v>217</v>
       </c>
-      <c r="I401" s="162" t="s">
+      <c r="I401" s="136" t="s">
         <v>206</v>
       </c>
-      <c r="J401" s="163" t="s">
+      <c r="J401" s="133" t="s">
         <v>236</v>
       </c>
     </row>
@@ -17074,13 +17073,13 @@
       <c r="G402" s="135">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H402" s="163" t="s">
+      <c r="H402" s="133" t="s">
         <v>217</v>
       </c>
-      <c r="I402" s="162" t="s">
+      <c r="I402" s="136" t="s">
         <v>238</v>
       </c>
-      <c r="J402" s="163" t="s">
+      <c r="J402" s="133" t="s">
         <v>223</v>
       </c>
     </row>
@@ -17106,13 +17105,13 @@
       <c r="G403" s="135">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H403" s="163" t="s">
+      <c r="H403" s="133" t="s">
         <v>217</v>
       </c>
-      <c r="I403" s="162" t="s">
+      <c r="I403" s="136" t="s">
         <v>240</v>
       </c>
-      <c r="J403" s="163" t="s">
+      <c r="J403" s="133" t="s">
         <v>241</v>
       </c>
     </row>
@@ -17138,13 +17137,13 @@
       <c r="G404" s="135">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H404" s="163" t="s">
+      <c r="H404" s="133" t="s">
         <v>217</v>
       </c>
-      <c r="I404" s="162" t="s">
+      <c r="I404" s="136" t="s">
         <v>243</v>
       </c>
-      <c r="J404" s="163" t="s">
+      <c r="J404" s="133" t="s">
         <v>244</v>
       </c>
     </row>
@@ -17170,13 +17169,13 @@
       <c r="G405" s="135">
         <v>0.48958333333333331</v>
       </c>
-      <c r="H405" s="163" t="s">
+      <c r="H405" s="133" t="s">
         <v>205</v>
       </c>
-      <c r="I405" s="162" t="s">
+      <c r="I405" s="136" t="s">
         <v>206</v>
       </c>
-      <c r="J405" s="163"/>
+      <c r="J405" s="133"/>
     </row>
     <row r="406" spans="1:10">
       <c r="A406" s="133" t="s">
@@ -17200,13 +17199,13 @@
       <c r="G406" s="135">
         <v>0.63541666666666663</v>
       </c>
-      <c r="H406" s="163" t="s">
+      <c r="H406" s="133" t="s">
         <v>247</v>
       </c>
-      <c r="I406" s="162" t="s">
+      <c r="I406" s="136" t="s">
         <v>206</v>
       </c>
-      <c r="J406" s="163"/>
+      <c r="J406" s="133"/>
     </row>
     <row r="407" spans="1:10">
       <c r="A407" s="133" t="s">
@@ -17230,13 +17229,13 @@
       <c r="G407" s="135">
         <v>0.69791666666666663</v>
       </c>
-      <c r="H407" s="163" t="s">
+      <c r="H407" s="133" t="s">
         <v>247</v>
       </c>
-      <c r="I407" s="162" t="s">
+      <c r="I407" s="136" t="s">
         <v>206</v>
       </c>
-      <c r="J407" s="163"/>
+      <c r="J407" s="133"/>
     </row>
     <row r="408" spans="1:10">
       <c r="A408" s="137" t="s">
@@ -17260,13 +17259,13 @@
       <c r="G408" s="139">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H408" s="164" t="s">
+      <c r="H408" s="137" t="s">
         <v>251</v>
       </c>
-      <c r="I408" s="164" t="s">
+      <c r="I408" s="137" t="s">
         <v>213</v>
       </c>
-      <c r="J408" s="164" t="s">
+      <c r="J408" s="137" t="s">
         <v>252</v>
       </c>
     </row>
@@ -17292,13 +17291,13 @@
       <c r="G409" s="139">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H409" s="164" t="s">
+      <c r="H409" s="137" t="s">
         <v>251</v>
       </c>
-      <c r="I409" s="165" t="s">
+      <c r="I409" s="160" t="s">
         <v>253</v>
       </c>
-      <c r="J409" s="165" t="s">
+      <c r="J409" s="160" t="s">
         <v>240</v>
       </c>
     </row>
@@ -17324,13 +17323,13 @@
       <c r="G410" s="139">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H410" s="164" t="s">
+      <c r="H410" s="137" t="s">
         <v>251</v>
       </c>
-      <c r="I410" s="164" t="s">
+      <c r="I410" s="137" t="s">
         <v>213</v>
       </c>
-      <c r="J410" s="164"/>
+      <c r="J410" s="137"/>
     </row>
     <row r="411" spans="1:10">
       <c r="A411" s="137" t="s">
@@ -17354,13 +17353,13 @@
       <c r="G411" s="139">
         <v>0.61458333333333337</v>
       </c>
-      <c r="H411" s="164" t="s">
+      <c r="H411" s="137" t="s">
         <v>214</v>
       </c>
-      <c r="I411" s="164" t="s">
+      <c r="I411" s="137" t="s">
         <v>213</v>
       </c>
-      <c r="J411" s="165"/>
+      <c r="J411" s="160"/>
     </row>
     <row r="412" spans="1:10">
       <c r="A412" s="137" t="s">
@@ -17384,13 +17383,13 @@
       <c r="G412" s="139">
         <v>0.61458333333333337</v>
       </c>
-      <c r="H412" s="164" t="s">
+      <c r="H412" s="137" t="s">
         <v>258</v>
       </c>
-      <c r="I412" s="164" t="s">
+      <c r="I412" s="137" t="s">
         <v>213</v>
       </c>
-      <c r="J412" s="165"/>
+      <c r="J412" s="160"/>
     </row>
     <row r="413" spans="1:10" ht="15">
       <c r="A413" s="137" t="s">
@@ -17414,13 +17413,13 @@
       <c r="G413" s="139">
         <v>0.48958333333333331</v>
       </c>
-      <c r="H413" s="164" t="s">
+      <c r="H413" s="137" t="s">
         <v>258</v>
       </c>
-      <c r="I413" s="164" t="s">
+      <c r="I413" s="137" t="s">
         <v>241</v>
       </c>
-      <c r="J413" s="164"/>
+      <c r="J413" s="137"/>
     </row>
     <row r="414" spans="1:10" ht="15">
       <c r="A414" s="137" t="s">
@@ -17444,13 +17443,13 @@
       <c r="G414" s="139">
         <v>0.48958333333333331</v>
       </c>
-      <c r="H414" s="164" t="s">
+      <c r="H414" s="137" t="s">
         <v>258</v>
       </c>
-      <c r="I414" s="164" t="s">
+      <c r="I414" s="137" t="s">
         <v>241</v>
       </c>
-      <c r="J414" s="165"/>
+      <c r="J414" s="160"/>
     </row>
     <row r="415" spans="1:10">
       <c r="A415" s="137" t="s">
@@ -17474,13 +17473,13 @@
       <c r="G415" s="139">
         <v>0.55208333333333337</v>
       </c>
-      <c r="H415" s="164" t="s">
+      <c r="H415" s="137" t="s">
         <v>214</v>
       </c>
-      <c r="I415" s="166" t="s">
+      <c r="I415" s="161" t="s">
         <v>240</v>
       </c>
-      <c r="J415" s="165"/>
+      <c r="J415" s="160"/>
     </row>
     <row r="416" spans="1:10" ht="15">
       <c r="A416" s="137" t="s">
@@ -17504,13 +17503,13 @@
       <c r="G416" s="139">
         <v>0.55208333333333337</v>
       </c>
-      <c r="H416" s="164" t="s">
+      <c r="H416" s="137" t="s">
         <v>214</v>
       </c>
-      <c r="I416" s="166" t="s">
+      <c r="I416" s="161" t="s">
         <v>240</v>
       </c>
-      <c r="J416" s="165"/>
+      <c r="J416" s="160"/>
     </row>
     <row r="417" spans="1:10" ht="15">
       <c r="A417" s="137" t="s">
@@ -17534,13 +17533,13 @@
       <c r="G417" s="139">
         <v>0.55208333333333337</v>
       </c>
-      <c r="H417" s="164" t="s">
+      <c r="H417" s="137" t="s">
         <v>214</v>
       </c>
-      <c r="I417" s="166" t="s">
+      <c r="I417" s="161" t="s">
         <v>240</v>
       </c>
-      <c r="J417" s="165"/>
+      <c r="J417" s="160"/>
     </row>
     <row r="418" spans="1:10">
       <c r="A418" s="137" t="s">
@@ -17564,13 +17563,13 @@
       <c r="G418" s="139">
         <v>0.73958333333333337</v>
       </c>
-      <c r="H418" s="164" t="s">
+      <c r="H418" s="137" t="s">
         <v>266</v>
       </c>
-      <c r="I418" s="164" t="s">
+      <c r="I418" s="137" t="s">
         <v>214</v>
       </c>
-      <c r="J418" s="164" t="s">
+      <c r="J418" s="137" t="s">
         <v>213</v>
       </c>
     </row>
@@ -17596,13 +17595,13 @@
       <c r="G419" s="139">
         <v>0.73958333333333337</v>
       </c>
-      <c r="H419" s="164" t="s">
+      <c r="H419" s="137" t="s">
         <v>266</v>
       </c>
-      <c r="I419" s="164" t="s">
+      <c r="I419" s="137" t="s">
         <v>214</v>
       </c>
-      <c r="J419" s="164" t="s">
+      <c r="J419" s="137" t="s">
         <v>213</v>
       </c>
     </row>
@@ -17628,13 +17627,13 @@
       <c r="G420" s="139">
         <v>0.73958333333333337</v>
       </c>
-      <c r="H420" s="164" t="s">
+      <c r="H420" s="137" t="s">
         <v>266</v>
       </c>
-      <c r="I420" s="164" t="s">
+      <c r="I420" s="137" t="s">
         <v>214</v>
       </c>
-      <c r="J420" s="164" t="s">
+      <c r="J420" s="137" t="s">
         <v>213</v>
       </c>
     </row>
@@ -17660,13 +17659,13 @@
       <c r="G421" s="139">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H421" s="166" t="s">
+      <c r="H421" s="161" t="s">
         <v>271</v>
       </c>
-      <c r="I421" s="164" t="s">
+      <c r="I421" s="137" t="s">
         <v>272</v>
       </c>
-      <c r="J421" s="165"/>
+      <c r="J421" s="160"/>
     </row>
     <row r="422" spans="1:10">
       <c r="A422" s="137" t="s">
@@ -17690,13 +17689,13 @@
       <c r="G422" s="139">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H422" s="166" t="s">
+      <c r="H422" s="161" t="s">
         <v>271</v>
       </c>
-      <c r="I422" s="164" t="s">
+      <c r="I422" s="137" t="s">
         <v>272</v>
       </c>
-      <c r="J422" s="165"/>
+      <c r="J422" s="160"/>
     </row>
     <row r="423" spans="1:10">
       <c r="A423" s="137" t="s">
@@ -17720,13 +17719,13 @@
       <c r="G423" s="139">
         <v>0.48958333333333331</v>
       </c>
-      <c r="H423" s="166" t="s">
+      <c r="H423" s="161" t="s">
         <v>271</v>
       </c>
-      <c r="I423" s="164" t="s">
+      <c r="I423" s="137" t="s">
         <v>272</v>
       </c>
-      <c r="J423" s="165"/>
+      <c r="J423" s="160"/>
     </row>
     <row r="424" spans="1:10">
       <c r="A424" s="137" t="s">
@@ -17750,13 +17749,13 @@
       <c r="G424" s="139">
         <v>0.55208333333333337</v>
       </c>
-      <c r="H424" s="164" t="s">
+      <c r="H424" s="137" t="s">
         <v>266</v>
       </c>
-      <c r="I424" s="165" t="s">
+      <c r="I424" s="160" t="s">
         <v>276</v>
       </c>
-      <c r="J424" s="165" t="s">
+      <c r="J424" s="160" t="s">
         <v>277</v>
       </c>
     </row>
@@ -17782,13 +17781,13 @@
       <c r="G425" s="139">
         <v>0.55208333333333337</v>
       </c>
-      <c r="H425" s="164" t="s">
+      <c r="H425" s="137" t="s">
         <v>266</v>
       </c>
-      <c r="I425" s="165" t="s">
+      <c r="I425" s="160" t="s">
         <v>276</v>
       </c>
-      <c r="J425" s="165" t="s">
+      <c r="J425" s="160" t="s">
         <v>277</v>
       </c>
     </row>
@@ -17814,13 +17813,13 @@
       <c r="G426" s="139">
         <v>0.61458333333333337</v>
       </c>
-      <c r="H426" s="164" t="s">
+      <c r="H426" s="137" t="s">
         <v>271</v>
       </c>
-      <c r="I426" s="165" t="s">
+      <c r="I426" s="160" t="s">
         <v>231</v>
       </c>
-      <c r="J426" s="165" t="s">
+      <c r="J426" s="160" t="s">
         <v>280</v>
       </c>
     </row>
@@ -17846,13 +17845,13 @@
       <c r="G427" s="139">
         <v>0.61458333333333337</v>
       </c>
-      <c r="H427" s="164" t="s">
+      <c r="H427" s="137" t="s">
         <v>271</v>
       </c>
-      <c r="I427" s="166" t="s">
+      <c r="I427" s="161" t="s">
         <v>266</v>
       </c>
-      <c r="J427" s="165" t="s">
+      <c r="J427" s="160" t="s">
         <v>277</v>
       </c>
     </row>
@@ -17878,13 +17877,13 @@
       <c r="G428" s="139">
         <v>0.61458333333333337</v>
       </c>
-      <c r="H428" s="164" t="s">
+      <c r="H428" s="137" t="s">
         <v>271</v>
       </c>
-      <c r="I428" s="164" t="s">
+      <c r="I428" s="137" t="s">
         <v>213</v>
       </c>
-      <c r="J428" s="165" t="s">
+      <c r="J428" s="160" t="s">
         <v>272</v>
       </c>
     </row>
@@ -17910,13 +17909,13 @@
       <c r="G429" s="139">
         <v>0.61458333333333337</v>
       </c>
-      <c r="H429" s="164" t="s">
+      <c r="H429" s="137" t="s">
         <v>272</v>
       </c>
-      <c r="I429" s="164" t="s">
+      <c r="I429" s="137" t="s">
         <v>213</v>
       </c>
-      <c r="J429" s="165"/>
+      <c r="J429" s="160"/>
     </row>
     <row r="430" spans="1:10">
       <c r="A430" s="137" t="s">
@@ -17940,13 +17939,13 @@
       <c r="G430" s="139">
         <v>0.48958333333333331</v>
       </c>
-      <c r="H430" s="164" t="s">
+      <c r="H430" s="137" t="s">
         <v>283</v>
       </c>
-      <c r="I430" s="164" t="s">
+      <c r="I430" s="137" t="s">
         <v>214</v>
       </c>
-      <c r="J430" s="164" t="s">
+      <c r="J430" s="137" t="s">
         <v>271</v>
       </c>
     </row>
@@ -17972,13 +17971,13 @@
       <c r="G431" s="139">
         <v>0.48958333333333331</v>
       </c>
-      <c r="H431" s="164" t="s">
+      <c r="H431" s="137" t="s">
         <v>283</v>
       </c>
-      <c r="I431" s="164" t="s">
+      <c r="I431" s="137" t="s">
         <v>206</v>
       </c>
-      <c r="J431" s="164" t="s">
+      <c r="J431" s="137" t="s">
         <v>284</v>
       </c>
     </row>
@@ -18004,13 +18003,13 @@
       <c r="G432" s="139">
         <v>0.48958333333333331</v>
       </c>
-      <c r="H432" s="164" t="s">
+      <c r="H432" s="137" t="s">
         <v>283</v>
       </c>
-      <c r="I432" s="164" t="s">
+      <c r="I432" s="137" t="s">
         <v>285</v>
       </c>
-      <c r="J432" s="164" t="s">
+      <c r="J432" s="137" t="s">
         <v>240</v>
       </c>
     </row>
@@ -18036,13 +18035,13 @@
       <c r="G433" s="139">
         <v>0.48958333333333331</v>
       </c>
-      <c r="H433" s="164" t="s">
+      <c r="H433" s="137" t="s">
         <v>287</v>
       </c>
-      <c r="I433" s="164" t="s">
+      <c r="I433" s="137" t="s">
         <v>213</v>
       </c>
-      <c r="J433" s="165"/>
+      <c r="J433" s="160"/>
     </row>
     <row r="434" spans="1:10">
       <c r="A434" s="137" t="s">
@@ -18066,13 +18065,13 @@
       <c r="G434" s="139">
         <v>0.67708333333333337</v>
       </c>
-      <c r="H434" s="164" t="s">
+      <c r="H434" s="137" t="s">
         <v>214</v>
       </c>
-      <c r="I434" s="164" t="s">
+      <c r="I434" s="137" t="s">
         <v>251</v>
       </c>
-      <c r="J434" s="164"/>
+      <c r="J434" s="137"/>
     </row>
     <row r="435" spans="1:10">
       <c r="A435" s="137" t="s">
@@ -18096,13 +18095,13 @@
       <c r="G435" s="139">
         <v>0.73958333333333337</v>
       </c>
-      <c r="H435" s="164" t="s">
+      <c r="H435" s="137" t="s">
         <v>272</v>
       </c>
-      <c r="I435" s="164" t="s">
+      <c r="I435" s="137" t="s">
         <v>213</v>
       </c>
-      <c r="J435" s="165"/>
+      <c r="J435" s="160"/>
     </row>
     <row r="436" spans="1:10" ht="15">
       <c r="A436" s="137" t="s">
@@ -18126,13 +18125,13 @@
       <c r="G436" s="139">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H436" s="164" t="s">
+      <c r="H436" s="137" t="s">
         <v>217</v>
       </c>
-      <c r="I436" s="164" t="s">
+      <c r="I436" s="137" t="s">
         <v>213</v>
       </c>
-      <c r="J436" s="167" t="s">
+      <c r="J436" s="152" t="s">
         <v>291</v>
       </c>
     </row>
@@ -18158,13 +18157,13 @@
       <c r="G437" s="139">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H437" s="164" t="s">
+      <c r="H437" s="137" t="s">
         <v>217</v>
       </c>
-      <c r="I437" s="165" t="s">
+      <c r="I437" s="160" t="s">
         <v>292</v>
       </c>
-      <c r="J437" s="165" t="s">
+      <c r="J437" s="160" t="s">
         <v>210</v>
       </c>
     </row>
@@ -18190,13 +18189,13 @@
       <c r="G438" s="139">
         <v>0.48958333333333331</v>
       </c>
-      <c r="H438" s="164" t="s">
+      <c r="H438" s="137" t="s">
         <v>295</v>
       </c>
-      <c r="I438" s="164" t="s">
+      <c r="I438" s="137" t="s">
         <v>213</v>
       </c>
-      <c r="J438" s="165" t="s">
+      <c r="J438" s="160" t="s">
         <v>296</v>
       </c>
     </row>
@@ -18222,13 +18221,13 @@
       <c r="G439" s="139">
         <v>0.48958333333333331</v>
       </c>
-      <c r="H439" s="164" t="s">
+      <c r="H439" s="137" t="s">
         <v>295</v>
       </c>
-      <c r="I439" s="164" t="s">
+      <c r="I439" s="137" t="s">
         <v>285</v>
       </c>
-      <c r="J439" s="165" t="s">
+      <c r="J439" s="160" t="s">
         <v>210</v>
       </c>
     </row>
@@ -18254,13 +18253,13 @@
       <c r="G440" s="139">
         <v>0.48958333333333331</v>
       </c>
-      <c r="H440" s="164" t="s">
+      <c r="H440" s="137" t="s">
         <v>295</v>
       </c>
-      <c r="I440" s="164" t="s">
+      <c r="I440" s="137" t="s">
         <v>285</v>
       </c>
-      <c r="J440" s="165" t="s">
+      <c r="J440" s="160" t="s">
         <v>210</v>
       </c>
     </row>
@@ -19546,12 +19545,12 @@
         <v>372</v>
       </c>
       <c r="J482" s="152" t="s">
-        <v>291</v>
+        <v>373</v>
       </c>
     </row>
     <row r="483" spans="1:10">
       <c r="A483" s="140" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B483" s="140">
         <v>1</v>
@@ -19572,7 +19571,7 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H483" s="143" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="I483" s="148" t="s">
         <v>331</v>
@@ -19581,7 +19580,7 @@
     </row>
     <row r="484" spans="1:10" ht="15">
       <c r="A484" s="140" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B484" s="140">
         <v>1</v>
@@ -19590,7 +19589,7 @@
         <v>12</v>
       </c>
       <c r="D484" s="140" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E484" s="141">
         <v>46337</v>
@@ -19611,16 +19610,16 @@
     </row>
     <row r="485" spans="1:10" ht="15">
       <c r="A485" s="140" t="s">
+        <v>378</v>
+      </c>
+      <c r="B485" s="140">
+        <v>1</v>
+      </c>
+      <c r="C485" s="140" t="s">
+        <v>12</v>
+      </c>
+      <c r="D485" s="140" t="s">
         <v>377</v>
-      </c>
-      <c r="B485" s="140">
-        <v>1</v>
-      </c>
-      <c r="C485" s="140" t="s">
-        <v>12</v>
-      </c>
-      <c r="D485" s="140" t="s">
-        <v>376</v>
       </c>
       <c r="E485" s="141">
         <v>46337</v>
@@ -19643,7 +19642,7 @@
     </row>
     <row r="486" spans="1:10" ht="15">
       <c r="A486" s="140" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B486" s="140">
         <v>1</v>
@@ -19652,7 +19651,7 @@
         <v>12</v>
       </c>
       <c r="D486" s="140" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E486" s="141">
         <v>46337</v>
@@ -19675,7 +19674,7 @@
     </row>
     <row r="487" spans="1:10">
       <c r="A487" s="140" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B487" s="140">
         <v>1</v>
@@ -19705,7 +19704,7 @@
     </row>
     <row r="488" spans="1:10" ht="15">
       <c r="A488" s="140" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B488" s="140">
         <v>1</v>
@@ -19714,7 +19713,7 @@
         <v>12</v>
       </c>
       <c r="D488" s="140" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E488" s="141">
         <v>46337</v>
@@ -19726,7 +19725,7 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H488" s="143" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="I488" s="148" t="s">
         <v>331</v>
@@ -19737,7 +19736,7 @@
     </row>
     <row r="489" spans="1:10" ht="15">
       <c r="A489" s="140" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B489" s="140">
         <v>1</v>
@@ -19758,10 +19757,10 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H489" s="143" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="I489" s="151" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J489" s="151" t="s">
         <v>336</v>
@@ -19769,7 +19768,7 @@
     </row>
     <row r="490" spans="1:10" ht="15">
       <c r="A490" s="140" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B490" s="140">
         <v>1</v>
@@ -19778,7 +19777,7 @@
         <v>12</v>
       </c>
       <c r="D490" s="140" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E490" s="141">
         <v>46338</v>
@@ -19796,12 +19795,12 @@
         <v>331</v>
       </c>
       <c r="J490" s="151" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="491" spans="1:10" ht="15">
       <c r="A491" s="140" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B491" s="140">
         <v>1</v>
@@ -19833,7 +19832,7 @@
     </row>
     <row r="492" spans="1:10">
       <c r="A492" s="140" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B492" s="140">
         <v>1</v>
@@ -19842,7 +19841,7 @@
         <v>12</v>
       </c>
       <c r="D492" s="140" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E492" s="141">
         <v>46338</v>
@@ -19854,7 +19853,7 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H492" s="143" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="I492" s="148" t="s">
         <v>337</v>
@@ -19863,7 +19862,7 @@
     </row>
     <row r="493" spans="1:10" ht="15">
       <c r="A493" s="140" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B493" s="140">
         <v>1</v>
@@ -19895,7 +19894,7 @@
     </row>
     <row r="494" spans="1:10" ht="15">
       <c r="A494" s="140" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B494" s="140">
         <v>1</v>
@@ -19904,7 +19903,7 @@
         <v>12</v>
       </c>
       <c r="D494" s="140" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E494" s="141">
         <v>46338</v>
@@ -19927,7 +19926,7 @@
     </row>
     <row r="495" spans="1:10" ht="15">
       <c r="A495" s="140" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B495" s="140">
         <v>1</v>
@@ -19950,7 +19949,7 @@
       <c r="H495" s="143" t="s">
         <v>351</v>
       </c>
-      <c r="I495" s="160" t="s">
+      <c r="I495" s="158" t="s">
         <v>364</v>
       </c>
       <c r="J495" s="148" t="s">
@@ -19959,7 +19958,7 @@
     </row>
     <row r="496" spans="1:10" ht="15">
       <c r="A496" s="140" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B496" s="140">
         <v>1</v>
@@ -19991,7 +19990,7 @@
     </row>
     <row r="497" spans="1:10" ht="15">
       <c r="A497" s="140" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B497" s="140">
         <v>1</v>
@@ -20023,7 +20022,7 @@
     </row>
     <row r="498" spans="1:10" ht="15">
       <c r="A498" s="140" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B498" s="140">
         <v>1</v>
@@ -20032,7 +20031,7 @@
         <v>12</v>
       </c>
       <c r="D498" s="140" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E498" s="141">
         <v>46338</v>
@@ -20044,7 +20043,7 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H498" s="143" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="I498" s="148" t="s">
         <v>331</v>
@@ -20055,7 +20054,7 @@
     </row>
     <row r="499" spans="1:10" ht="15">
       <c r="A499" s="140" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B499" s="140">
         <v>1</v>
@@ -20064,7 +20063,7 @@
         <v>12</v>
       </c>
       <c r="D499" s="140" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E499" s="141">
         <v>46338</v>
@@ -20076,7 +20075,7 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H499" s="143" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="I499" s="151" t="s">
         <v>345</v>
@@ -20087,7 +20086,7 @@
     </row>
     <row r="500" spans="1:10" ht="15">
       <c r="A500" s="140" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B500" s="140">
         <v>1</v>
@@ -20108,7 +20107,7 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H500" s="143" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="I500" s="151" t="s">
         <v>243</v>
@@ -20117,7 +20116,7 @@
     </row>
     <row r="501" spans="1:10" ht="15">
       <c r="A501" s="140" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B501" s="140">
         <v>1</v>
@@ -20138,7 +20137,7 @@
         <v>0.73958333333333337</v>
       </c>
       <c r="H501" s="143" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="I501" s="148" t="s">
         <v>331</v>
@@ -20149,7 +20148,7 @@
     </row>
     <row r="502" spans="1:10">
       <c r="A502" s="140" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B502" s="140">
         <v>1</v>
@@ -20158,7 +20157,7 @@
         <v>12</v>
       </c>
       <c r="D502" s="140" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E502" s="141">
         <v>46338</v>
@@ -20170,7 +20169,7 @@
         <v>0.73958333333333337</v>
       </c>
       <c r="H502" s="143" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="I502" s="148" t="s">
         <v>337</v>
@@ -20181,7 +20180,7 @@
     </row>
     <row r="503" spans="1:10" ht="30.75">
       <c r="A503" s="140" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B503" s="140">
         <v>1</v>
@@ -20190,7 +20189,7 @@
         <v>12</v>
       </c>
       <c r="D503" s="140" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E503" s="141">
         <v>46339</v>
@@ -20204,8 +20203,8 @@
       <c r="H503" s="143" t="s">
         <v>217</v>
       </c>
-      <c r="I503" s="157" t="s">
-        <v>400</v>
+      <c r="I503" s="155" t="s">
+        <v>401</v>
       </c>
       <c r="J503" s="154" t="s">
         <v>347</v>
@@ -20213,7 +20212,7 @@
     </row>
     <row r="504" spans="1:10" ht="15">
       <c r="A504" s="140" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B504" s="140">
         <v>1</v>
@@ -20222,7 +20221,7 @@
         <v>12</v>
       </c>
       <c r="D504" s="140" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E504" s="141">
         <v>46339</v>
@@ -20245,7 +20244,7 @@
     </row>
     <row r="505" spans="1:10" ht="15">
       <c r="A505" s="140" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B505" s="140">
         <v>1</v>
@@ -20275,7 +20274,7 @@
     </row>
     <row r="506" spans="1:10">
       <c r="A506" s="140" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B506" s="140">
         <v>1</v>
@@ -20284,7 +20283,7 @@
         <v>12</v>
       </c>
       <c r="D506" s="140" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E506" s="141">
         <v>46339</v>
@@ -20307,7 +20306,7 @@
     </row>
     <row r="507" spans="1:10" ht="15">
       <c r="A507" s="140" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B507" s="140">
         <v>1</v>
@@ -20339,7 +20338,7 @@
     </row>
     <row r="508" spans="1:10">
       <c r="A508" s="140" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B508" s="140">
         <v>1</v>
@@ -20371,7 +20370,7 @@
     </row>
     <row r="509" spans="1:10" ht="15">
       <c r="A509" s="140" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B509" s="140">
         <v>1</v>
@@ -20403,7 +20402,7 @@
     </row>
     <row r="510" spans="1:10">
       <c r="A510" s="140" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B510" s="140">
         <v>1</v>
@@ -20430,12 +20429,12 @@
         <v>331</v>
       </c>
       <c r="J510" s="148" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="511" spans="1:10" ht="15">
       <c r="A511" s="140" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B511" s="140">
         <v>1</v>
@@ -20444,7 +20443,7 @@
         <v>12</v>
       </c>
       <c r="D511" s="140" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E511" s="141">
         <v>46339</v>
@@ -20458,8 +20457,8 @@
       <c r="H511" s="143" t="s">
         <v>345</v>
       </c>
-      <c r="I511" s="160" t="s">
-        <v>408</v>
+      <c r="I511" s="158" t="s">
+        <v>409</v>
       </c>
       <c r="J511" s="148" t="s">
         <v>334</v>
@@ -20467,7 +20466,7 @@
     </row>
     <row r="512" spans="1:10">
       <c r="A512" s="140" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B512" s="140">
         <v>1</v>
@@ -20476,7 +20475,7 @@
         <v>12</v>
       </c>
       <c r="D512" s="140" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E512" s="141">
         <v>46339</v>
@@ -20499,7 +20498,7 @@
     </row>
     <row r="513" spans="1:10">
       <c r="A513" s="140" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B513" s="140">
         <v>1</v>
@@ -20508,7 +20507,7 @@
         <v>12</v>
       </c>
       <c r="D513" s="140" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="E513" s="141">
         <v>46339</v>
@@ -20531,7 +20530,7 @@
     </row>
     <row r="514" spans="1:10" ht="15">
       <c r="A514" s="140" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B514" s="140">
         <v>1</v>
@@ -20540,7 +20539,7 @@
         <v>12</v>
       </c>
       <c r="D514" s="140" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="E514" s="141">
         <v>46339</v>
@@ -20563,7 +20562,7 @@
     </row>
     <row r="515" spans="1:10">
       <c r="A515" s="140" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B515" s="140">
         <v>1</v>
@@ -20572,7 +20571,7 @@
         <v>12</v>
       </c>
       <c r="D515" s="140" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="E515" s="141">
         <v>46339</v>
@@ -20590,12 +20589,12 @@
         <v>363</v>
       </c>
       <c r="J515" s="148" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="516" spans="1:10">
       <c r="A516" s="115" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B516" s="115">
         <v>1</v>
@@ -20616,7 +20615,7 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H516" s="115" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="I516" s="115" t="s">
         <v>253</v>
@@ -20627,7 +20626,7 @@
     </row>
     <row r="517" spans="1:10">
       <c r="A517" s="115" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B517" s="115">
         <v>1</v>
@@ -20648,18 +20647,18 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H517" s="115" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="I517" s="115" t="s">
         <v>240</v>
       </c>
       <c r="J517" s="115" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
     </row>
     <row r="518" spans="1:10">
       <c r="A518" s="115" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B518" s="115">
         <v>2</v>
@@ -20680,7 +20679,7 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H518" s="115" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="I518" s="115" t="s">
         <v>253</v>
@@ -20691,7 +20690,7 @@
     </row>
     <row r="519" spans="1:10">
       <c r="A519" s="115" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B519" s="115">
         <v>2</v>
@@ -20712,18 +20711,18 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H519" s="115" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="I519" s="115" t="s">
         <v>240</v>
       </c>
       <c r="J519" s="115" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
     </row>
     <row r="520" spans="1:10">
       <c r="A520" s="115" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B520" s="115">
         <v>1</v>
@@ -20744,7 +20743,7 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H520" s="115" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="I520" s="115" t="s">
         <v>253</v>
@@ -20755,7 +20754,7 @@
     </row>
     <row r="521" spans="1:10">
       <c r="A521" s="115" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B521" s="115">
         <v>1</v>
@@ -20776,18 +20775,18 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H521" s="115" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="I521" s="115" t="s">
         <v>240</v>
       </c>
       <c r="J521" s="115" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
     </row>
     <row r="522" spans="1:10">
       <c r="A522" s="115" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B522" s="115">
         <v>1</v>
@@ -20808,7 +20807,7 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H522" s="115" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="I522" s="115" t="s">
         <v>253</v>
@@ -20819,7 +20818,7 @@
     </row>
     <row r="523" spans="1:10">
       <c r="A523" s="115" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B523" s="115">
         <v>1</v>
@@ -20828,7 +20827,7 @@
         <v>12</v>
       </c>
       <c r="D523" s="115" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="E523" s="116">
         <v>46335</v>
@@ -20840,7 +20839,7 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H523" s="115" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="I523" s="115" t="s">
         <v>240</v>
@@ -20851,7 +20850,7 @@
     </row>
     <row r="524" spans="1:10">
       <c r="A524" s="115" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B524" s="115">
         <v>1</v>
@@ -20860,7 +20859,7 @@
         <v>12</v>
       </c>
       <c r="D524" s="115" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="E524" s="116">
         <v>46335</v>
@@ -20872,7 +20871,7 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H524" s="115" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="I524" s="115" t="s">
         <v>351</v>
@@ -20883,7 +20882,7 @@
     </row>
     <row r="525" spans="1:10">
       <c r="A525" s="115" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B525" s="115">
         <v>3</v>
@@ -20892,7 +20891,7 @@
         <v>12</v>
       </c>
       <c r="D525" s="115" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="E525" s="116">
         <v>46335</v>
@@ -20904,7 +20903,7 @@
         <v>0.61458333333333337</v>
       </c>
       <c r="H525" s="115" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="I525" s="115" t="s">
         <v>253</v>
@@ -20915,7 +20914,7 @@
     </row>
     <row r="526" spans="1:10">
       <c r="A526" s="115" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B526" s="115">
         <v>3</v>
@@ -20924,7 +20923,7 @@
         <v>12</v>
       </c>
       <c r="D526" s="115" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="E526" s="116">
         <v>46335</v>
@@ -20936,18 +20935,18 @@
         <v>0.61458333333333337</v>
       </c>
       <c r="H526" s="115" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="I526" s="115" t="s">
         <v>240</v>
       </c>
       <c r="J526" s="115" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="527" spans="1:10">
       <c r="A527" s="115" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B527" s="115">
         <v>1</v>
@@ -20956,7 +20955,7 @@
         <v>12</v>
       </c>
       <c r="D527" s="115" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E527" s="116">
         <v>46335</v>
@@ -20968,7 +20967,7 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H527" s="115" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="I527" s="115" t="s">
         <v>217</v>
@@ -20979,7 +20978,7 @@
     </row>
     <row r="528" spans="1:10">
       <c r="A528" s="115" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B528" s="115">
         <v>1</v>
@@ -20988,7 +20987,7 @@
         <v>12</v>
       </c>
       <c r="D528" s="115" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="E528" s="116">
         <v>46335</v>
@@ -21000,7 +20999,7 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H528" s="115" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="I528" s="115" t="s">
         <v>240</v>
@@ -21011,7 +21010,7 @@
     </row>
     <row r="529" spans="1:10">
       <c r="A529" s="115" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B529" s="115">
         <v>1</v>
@@ -21020,7 +21019,7 @@
         <v>12</v>
       </c>
       <c r="D529" s="115" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E529" s="116">
         <v>46336</v>
@@ -21032,7 +21031,7 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="H529" s="115" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="I529" s="115" t="s">
         <v>253</v>
@@ -21043,7 +21042,7 @@
     </row>
     <row r="530" spans="1:10">
       <c r="A530" s="115" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B530" s="115">
         <v>2</v>
@@ -21052,7 +21051,7 @@
         <v>12</v>
       </c>
       <c r="D530" s="115" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E530" s="116">
         <v>46336</v>
@@ -21064,7 +21063,7 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="H530" s="115" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="I530" s="115" t="s">
         <v>253</v>
@@ -21075,7 +21074,7 @@
     </row>
     <row r="531" spans="1:10">
       <c r="A531" s="115" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B531" s="115">
         <v>1</v>
@@ -21084,7 +21083,7 @@
         <v>12</v>
       </c>
       <c r="D531" s="115" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E531" s="116">
         <v>46336</v>
@@ -21096,10 +21095,10 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H531" s="115" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="I531" s="115" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="J531" s="115" t="s">
         <v>296</v>
@@ -21107,7 +21106,7 @@
     </row>
     <row r="532" spans="1:10">
       <c r="A532" s="115" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B532" s="115">
         <v>1</v>
@@ -21116,7 +21115,7 @@
         <v>12</v>
       </c>
       <c r="D532" s="115" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E532" s="116">
         <v>46336</v>
@@ -21128,10 +21127,10 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H532" s="115" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="I532" s="115" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="J532" s="115" t="s">
         <v>296</v>
@@ -21139,7 +21138,7 @@
     </row>
     <row r="533" spans="1:10">
       <c r="A533" s="115" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B533" s="115">
         <v>1</v>
@@ -21148,7 +21147,7 @@
         <v>12</v>
       </c>
       <c r="D533" s="115" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="E533" s="116">
         <v>46336</v>
@@ -21160,10 +21159,10 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H533" s="115" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="I533" s="115" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="J533" s="115" t="s">
         <v>361</v>
@@ -21171,7 +21170,7 @@
     </row>
     <row r="534" spans="1:10">
       <c r="A534" s="115" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B534" s="115">
         <v>1</v>
@@ -21180,7 +21179,7 @@
         <v>12</v>
       </c>
       <c r="D534" s="115" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="E534" s="116">
         <v>46336</v>
@@ -21192,10 +21191,10 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H534" s="115" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="I534" s="115" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="J534" s="115" t="s">
         <v>370</v>
@@ -21203,7 +21202,7 @@
     </row>
     <row r="535" spans="1:10">
       <c r="A535" s="115" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B535" s="115">
         <v>1</v>
@@ -21212,7 +21211,7 @@
         <v>12</v>
       </c>
       <c r="D535" s="115" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="E535" s="116">
         <v>46336</v>
@@ -21224,18 +21223,18 @@
         <v>0.61458333333333337</v>
       </c>
       <c r="H535" s="115" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="I535" s="115" t="s">
         <v>210</v>
       </c>
       <c r="J535" s="115" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="536" spans="1:10">
       <c r="A536" s="115" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B536" s="115">
         <v>1</v>
@@ -21244,7 +21243,7 @@
         <v>12</v>
       </c>
       <c r="D536" s="115" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E536" s="116">
         <v>46336</v>
@@ -21256,18 +21255,18 @@
         <v>0.61458333333333337</v>
       </c>
       <c r="H536" s="115" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="I536" s="115" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="J536" s="115" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="537" spans="1:10">
       <c r="A537" s="115" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B537" s="115">
         <v>1</v>
@@ -21276,7 +21275,7 @@
         <v>12</v>
       </c>
       <c r="D537" s="115" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E537" s="116">
         <v>46336</v>
@@ -21288,7 +21287,7 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H537" s="115" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="I537" s="115" t="s">
         <v>253</v>
@@ -21299,7 +21298,7 @@
     </row>
     <row r="538" spans="1:10">
       <c r="A538" s="115" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B538" s="115">
         <v>1</v>
@@ -21308,7 +21307,7 @@
         <v>12</v>
       </c>
       <c r="D538" s="115" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E538" s="116">
         <v>46336</v>
@@ -21320,18 +21319,18 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H538" s="115" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="I538" s="115" t="s">
         <v>227</v>
       </c>
       <c r="J538" s="115" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="539" spans="1:10" ht="15">
       <c r="A539" s="115" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B539" s="115">
         <v>1</v>
@@ -21340,7 +21339,7 @@
         <v>12</v>
       </c>
       <c r="D539" s="115" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E539" s="116">
         <v>46337</v>
@@ -21352,16 +21351,16 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="H539" s="115" t="s">
-        <v>431</v>
-      </c>
-      <c r="I539" s="169" t="s">
+        <v>432</v>
+      </c>
+      <c r="I539" s="162" t="s">
         <v>243</v>
       </c>
       <c r="J539" s="115"/>
     </row>
     <row r="540" spans="1:10">
       <c r="A540" s="115" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B540" s="115">
         <v>1</v>
@@ -21370,7 +21369,7 @@
         <v>12</v>
       </c>
       <c r="D540" s="115" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E540" s="116">
         <v>46337</v>
@@ -21382,18 +21381,18 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="H540" s="115" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="I540" s="115" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="J540" s="115" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="541" spans="1:10">
       <c r="A541" s="115" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B541" s="115">
         <v>1</v>
@@ -21402,7 +21401,7 @@
         <v>12</v>
       </c>
       <c r="D541" s="115" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E541" s="116">
         <v>46337</v>
@@ -21414,18 +21413,18 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="H541" s="115" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="I541" s="115" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="J541" s="115" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="542" spans="1:10">
       <c r="A542" s="115" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B542" s="115">
         <v>1</v>
@@ -21434,7 +21433,7 @@
         <v>12</v>
       </c>
       <c r="D542" s="115" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E542" s="116">
         <v>46337</v>
@@ -21446,7 +21445,7 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H542" s="115" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="I542" s="115" t="s">
         <v>253</v>
@@ -21457,7 +21456,7 @@
     </row>
     <row r="543" spans="1:10">
       <c r="A543" s="115" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B543" s="115">
         <v>1</v>
@@ -21466,7 +21465,7 @@
         <v>12</v>
       </c>
       <c r="D543" s="115" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E543" s="116">
         <v>46337</v>
@@ -21478,18 +21477,18 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H543" s="115" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="I543" s="115" t="s">
         <v>287</v>
       </c>
       <c r="J543" s="115" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="544" spans="1:10">
       <c r="A544" s="115" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B544" s="115">
         <v>1</v>
@@ -21498,7 +21497,7 @@
         <v>12</v>
       </c>
       <c r="D544" s="115" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E544" s="116">
         <v>46337</v>
@@ -21516,12 +21515,12 @@
         <v>253</v>
       </c>
       <c r="J544" s="115" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="545" spans="1:10">
       <c r="A545" s="115" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B545" s="115">
         <v>1</v>
@@ -21530,7 +21529,7 @@
         <v>12</v>
       </c>
       <c r="D545" s="115" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E545" s="116">
         <v>46337</v>
@@ -21553,7 +21552,7 @@
     </row>
     <row r="546" spans="1:10">
       <c r="A546" s="115" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B546" s="115">
         <v>1</v>
@@ -21562,7 +21561,7 @@
         <v>12</v>
       </c>
       <c r="D546" s="115" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E546" s="116">
         <v>46337</v>
@@ -21580,12 +21579,12 @@
         <v>214</v>
       </c>
       <c r="J546" s="115" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="547" spans="1:10">
       <c r="A547" s="115" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B547" s="115">
         <v>1</v>
@@ -21606,7 +21605,7 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="H547" s="115" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="I547" s="115" t="s">
         <v>253</v>
@@ -21615,7 +21614,7 @@
     </row>
     <row r="548" spans="1:10">
       <c r="A548" s="115" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B548" s="115">
         <v>1</v>
@@ -21624,7 +21623,7 @@
         <v>12</v>
       </c>
       <c r="D548" s="115" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E548" s="116">
         <v>46338</v>
@@ -21636,7 +21635,7 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H548" s="115" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="I548" s="115" t="s">
         <v>253</v>
@@ -21647,7 +21646,7 @@
     </row>
     <row r="549" spans="1:10">
       <c r="A549" s="115" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B549" s="115">
         <v>1</v>
@@ -21668,7 +21667,7 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H549" s="115" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="I549" s="115" t="s">
         <v>352</v>
@@ -21679,7 +21678,7 @@
     </row>
     <row r="550" spans="1:10">
       <c r="A550" s="115" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B550" s="115">
         <v>1</v>
@@ -21688,7 +21687,7 @@
         <v>12</v>
       </c>
       <c r="D550" s="115" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="E550" s="116">
         <v>46338</v>
@@ -21700,7 +21699,7 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H550" s="115" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="I550" s="115" t="s">
         <v>296</v>
@@ -21711,7 +21710,7 @@
     </row>
     <row r="551" spans="1:10">
       <c r="A551" s="115" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B551" s="115">
         <v>1</v>
@@ -21720,7 +21719,7 @@
         <v>12</v>
       </c>
       <c r="D551" s="115" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E551" s="116">
         <v>46338</v>
@@ -21732,7 +21731,7 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H551" s="115" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="I551" s="115" t="s">
         <v>253</v>
@@ -21743,7 +21742,7 @@
     </row>
     <row r="552" spans="1:10">
       <c r="A552" s="115" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B552" s="115">
         <v>2</v>
@@ -21752,7 +21751,7 @@
         <v>12</v>
       </c>
       <c r="D552" s="115" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E552" s="116">
         <v>46338</v>
@@ -21764,7 +21763,7 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H552" s="115" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="I552" s="115" t="s">
         <v>253</v>
@@ -21775,7 +21774,7 @@
     </row>
     <row r="553" spans="1:10">
       <c r="A553" s="115" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B553" s="115">
         <v>1</v>
@@ -21784,7 +21783,7 @@
         <v>12</v>
       </c>
       <c r="D553" s="115" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="E553" s="116">
         <v>46338</v>
@@ -21796,7 +21795,7 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H553" s="115" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="I553" s="115" t="s">
         <v>253</v>
@@ -21807,7 +21806,7 @@
     </row>
     <row r="554" spans="1:10">
       <c r="A554" s="115" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B554" s="115">
         <v>1</v>
@@ -21816,7 +21815,7 @@
         <v>12</v>
       </c>
       <c r="D554" s="115" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="E554" s="116">
         <v>46338</v>
@@ -21828,18 +21827,18 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H554" s="115" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="I554" s="115" t="s">
         <v>240</v>
       </c>
       <c r="J554" s="115" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="555" spans="1:10">
       <c r="A555" s="115" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B555" s="115">
         <v>1</v>
@@ -21848,7 +21847,7 @@
         <v>12</v>
       </c>
       <c r="D555" s="115" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="E555" s="116">
         <v>46339</v>
@@ -21860,18 +21859,18 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H555" s="115" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="I555" s="115" t="s">
         <v>361</v>
       </c>
-      <c r="J555" s="168" t="s">
+      <c r="J555" s="115" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="556" spans="1:10">
       <c r="A556" s="115" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B556" s="115">
         <v>1</v>
@@ -21880,7 +21879,7 @@
         <v>12</v>
       </c>
       <c r="D556" s="115" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="E556" s="116">
         <v>46339</v>
@@ -21892,7 +21891,7 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H556" s="115" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="I556" s="115" t="s">
         <v>240</v>
@@ -21903,7 +21902,7 @@
     </row>
     <row r="557" spans="1:10">
       <c r="A557" s="115" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B557" s="115">
         <v>1</v>
@@ -21927,15 +21926,15 @@
         <v>266</v>
       </c>
       <c r="I557" s="115" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="J557" s="115" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="558" spans="1:10">
       <c r="A558" s="115" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B558" s="115">
         <v>1</v>
@@ -21944,7 +21943,7 @@
         <v>12</v>
       </c>
       <c r="D558" s="115" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E558" s="116">
         <v>46336</v>
@@ -21959,7 +21958,7 @@
         <v>266</v>
       </c>
       <c r="I558" s="115" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J558" s="115" t="s">
         <v>210</v>
@@ -21967,7 +21966,7 @@
     </row>
     <row r="559" spans="1:10">
       <c r="A559" s="115" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B559" s="115">
         <v>1</v>
@@ -21988,10 +21987,10 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H559" s="115" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="I559" s="115" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="J559" s="115" t="s">
         <v>223</v>
@@ -21999,7 +21998,7 @@
     </row>
     <row r="560" spans="1:10">
       <c r="A560" s="115" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B560" s="115">
         <v>1</v>
@@ -22020,7 +22019,7 @@
         <v>0.61458333333333337</v>
       </c>
       <c r="H560" s="115" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="I560" s="115" t="s">
         <v>285</v>
@@ -22029,7 +22028,7 @@
     </row>
     <row r="561" spans="1:10" ht="15">
       <c r="A561" s="115" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B561" s="115">
         <v>1</v>
@@ -22061,7 +22060,7 @@
     </row>
     <row r="562" spans="1:10">
       <c r="A562" s="115" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B562" s="115">
         <v>1</v>
@@ -22088,12 +22087,12 @@
         <v>240</v>
       </c>
       <c r="J562" s="152" t="s">
-        <v>291</v>
+        <v>477</v>
       </c>
     </row>
     <row r="563" spans="1:10">
       <c r="A563" s="115" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B563" s="115">
         <v>1</v>
@@ -22114,7 +22113,7 @@
         <v>0.61458333333333337</v>
       </c>
       <c r="H563" s="115" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="I563" s="115" t="s">
         <v>309</v>
@@ -22123,7 +22122,7 @@
     </row>
     <row r="564" spans="1:10">
       <c r="A564" s="115" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B564" s="115">
         <v>1</v>
@@ -22144,7 +22143,7 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H564" s="115" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="I564" s="115" t="s">
         <v>217</v>
@@ -22153,7 +22152,7 @@
     </row>
     <row r="565" spans="1:10">
       <c r="A565" s="115" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B565" s="115">
         <v>1</v>
@@ -22183,7 +22182,7 @@
     </row>
     <row r="566" spans="1:10">
       <c r="A566" s="115" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B566" s="115">
         <v>1</v>
@@ -22207,7 +22206,7 @@
         <v>210</v>
       </c>
       <c r="I566" s="152" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="J566" s="115" t="s">
         <v>266</v>
@@ -22215,7 +22214,7 @@
     </row>
     <row r="567" spans="1:10">
       <c r="A567" s="115" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B567" s="115">
         <v>1</v>
@@ -22239,15 +22238,15 @@
         <v>210</v>
       </c>
       <c r="I567" s="152" t="s">
-        <v>473</v>
-      </c>
-      <c r="J567" s="115" t="s">
-        <v>408</v>
+        <v>474</v>
+      </c>
+      <c r="J567" s="165" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="568" spans="1:10">
       <c r="A568" s="115" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B568" s="115">
         <v>1</v>
@@ -22279,7 +22278,7 @@
     </row>
     <row r="569" spans="1:10" ht="15">
       <c r="A569" s="115" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B569" s="115">
         <v>1</v>
@@ -22303,7 +22302,7 @@
         <v>217</v>
       </c>
       <c r="I569" s="130" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="J569" s="115" t="s">
         <v>296</v>
@@ -22311,7 +22310,7 @@
     </row>
     <row r="570" spans="1:10">
       <c r="A570" s="115" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B570" s="115">
         <v>1</v>
@@ -22320,7 +22319,7 @@
         <v>12</v>
       </c>
       <c r="D570" s="115" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="E570" s="116">
         <v>46339</v>
@@ -22341,7 +22340,7 @@
     </row>
     <row r="571" spans="1:10">
       <c r="A571" s="144" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B571" s="144">
         <v>1</v>
@@ -22350,7 +22349,7 @@
         <v>12</v>
       </c>
       <c r="D571" s="144" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E571" s="146">
         <v>46337</v>
@@ -22362,18 +22361,18 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="H571" s="144" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="I571" s="144" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="J571" s="144" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="572" spans="1:10">
       <c r="A572" s="144" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B572" s="144">
         <v>1</v>
@@ -22382,7 +22381,7 @@
         <v>12</v>
       </c>
       <c r="D572" s="144" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="E572" s="146">
         <v>46335</v>
@@ -22394,18 +22393,18 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H572" s="144" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="I572" s="144" t="s">
         <v>285</v>
       </c>
       <c r="J572" s="144" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="573" spans="1:10">
       <c r="A573" s="144" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B573" s="144">
         <v>1</v>
@@ -22414,7 +22413,7 @@
         <v>12</v>
       </c>
       <c r="D573" s="144" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="E573" s="146">
         <v>46335</v>
@@ -22426,7 +22425,7 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H573" s="144" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="I573" s="144" t="s">
         <v>213</v>
@@ -22435,7 +22434,7 @@
     </row>
     <row r="574" spans="1:10">
       <c r="A574" s="144" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B574" s="144">
         <v>1</v>
@@ -22456,18 +22455,18 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H574" s="144" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="I574" s="144" t="s">
         <v>347</v>
       </c>
       <c r="J574" s="144" t="s">
-        <v>490</v>
+        <v>477</v>
       </c>
     </row>
     <row r="575" spans="1:10" ht="15">
       <c r="A575" s="144" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B575" s="144">
         <v>1</v>
@@ -22476,7 +22475,7 @@
         <v>12</v>
       </c>
       <c r="D575" s="144" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="E575" s="146">
         <v>46339</v>
@@ -22488,12 +22487,12 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H575" s="144" t="s">
-        <v>440</v>
-      </c>
-      <c r="I575" s="144" t="s">
-        <v>492</v>
-      </c>
-      <c r="J575" s="161" t="s">
+        <v>441</v>
+      </c>
+      <c r="I575" s="152" t="s">
+        <v>291</v>
+      </c>
+      <c r="J575" s="159" t="s">
         <v>493</v>
       </c>
     </row>
@@ -22557,7 +22556,7 @@
         <v>497</v>
       </c>
       <c r="D579" s="119" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E579" s="120">
         <v>46335</v>
@@ -22569,7 +22568,7 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H579" s="119" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="I579" s="119" t="s">
         <v>206</v>
@@ -22586,7 +22585,7 @@
         <v>497</v>
       </c>
       <c r="D580" s="119" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E580" s="120">
         <v>46336</v>
@@ -22615,7 +22614,7 @@
         <v>497</v>
       </c>
       <c r="D581" s="119" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E581" s="120">
         <v>46337</v>
@@ -22644,7 +22643,7 @@
         <v>497</v>
       </c>
       <c r="D582" s="119" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E582" s="120">
         <v>46338</v>
@@ -22673,7 +22672,7 @@
         <v>497</v>
       </c>
       <c r="D583" s="122" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E583" s="123">
         <v>46335</v>
@@ -22685,9 +22684,9 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H583" s="122" t="s">
-        <v>488</v>
-      </c>
-      <c r="I583" s="158" t="s">
+        <v>490</v>
+      </c>
+      <c r="I583" s="156" t="s">
         <v>54</v>
       </c>
     </row>
@@ -22716,13 +22715,13 @@
       <c r="H584" s="122" t="s">
         <v>503</v>
       </c>
-      <c r="I584" s="159" t="s">
-        <v>504</v>
+      <c r="I584" s="157" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="585" spans="1:10" ht="15">
       <c r="A585" s="122" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B585" s="122">
         <v>1</v>
@@ -22731,7 +22730,7 @@
         <v>497</v>
       </c>
       <c r="D585" s="122" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E585" s="123">
         <v>46336</v>
@@ -22743,15 +22742,15 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H585" s="122" t="s">
-        <v>506</v>
-      </c>
-      <c r="I585" s="159" t="s">
+        <v>505</v>
+      </c>
+      <c r="I585" s="157" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="586" spans="1:10" ht="15">
       <c r="A586" s="122" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="B586" s="122">
         <v>1</v>
@@ -22772,15 +22771,15 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H586" s="122" t="s">
-        <v>508</v>
-      </c>
-      <c r="I586" s="159" t="s">
-        <v>504</v>
+        <v>507</v>
+      </c>
+      <c r="I586" s="157" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="587" spans="1:10" ht="15">
       <c r="A587" s="125" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="B587" s="125">
         <v>1</v>
@@ -22789,7 +22788,7 @@
         <v>497</v>
       </c>
       <c r="D587" s="125" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="E587" s="126">
         <v>46338</v>
@@ -22803,13 +22802,13 @@
       <c r="H587" s="125" t="s">
         <v>296</v>
       </c>
-      <c r="I587" s="158" t="s">
+      <c r="I587" s="156" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="588" spans="1:10" ht="15">
       <c r="A588" s="122" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B588" s="122">
         <v>1</v>
@@ -22818,7 +22817,7 @@
         <v>497</v>
       </c>
       <c r="D588" s="122" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E588" s="123">
         <v>46339</v>
@@ -22830,15 +22829,15 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H588" s="122" t="s">
+        <v>511</v>
+      </c>
+      <c r="I588" s="157" t="s">
         <v>512</v>
-      </c>
-      <c r="I588" s="159" t="s">
-        <v>513</v>
       </c>
     </row>
     <row r="589" spans="1:10" ht="15">
       <c r="A589" s="122" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B589" s="122">
         <v>1</v>
@@ -22847,7 +22846,7 @@
         <v>497</v>
       </c>
       <c r="D589" s="122" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E589" s="123">
         <v>46339</v>
@@ -22859,15 +22858,15 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H589" s="122" t="s">
+        <v>511</v>
+      </c>
+      <c r="I589" s="157" t="s">
         <v>512</v>
-      </c>
-      <c r="I589" s="159" t="s">
-        <v>513</v>
       </c>
     </row>
     <row r="590" spans="1:10" ht="15">
       <c r="A590" s="122" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B590" s="122">
         <v>1</v>
@@ -22876,7 +22875,7 @@
         <v>497</v>
       </c>
       <c r="D590" s="122" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E590" s="123">
         <v>46339</v>
@@ -22888,15 +22887,15 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H590" s="122" t="s">
+        <v>511</v>
+      </c>
+      <c r="I590" s="157" t="s">
         <v>512</v>
-      </c>
-      <c r="I590" s="159" t="s">
-        <v>513</v>
       </c>
     </row>
     <row r="591" spans="1:10" ht="15">
       <c r="A591" s="122" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B591" s="122">
         <v>1</v>
@@ -22905,7 +22904,7 @@
         <v>497</v>
       </c>
       <c r="D591" s="122" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E591" s="123">
         <v>46335</v>
@@ -22917,15 +22916,15 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H591" s="122" t="s">
-        <v>427</v>
-      </c>
-      <c r="I591" s="159" t="s">
-        <v>517</v>
+        <v>428</v>
+      </c>
+      <c r="I591" s="157" t="s">
+        <v>516</v>
       </c>
     </row>
     <row r="592" spans="1:10" ht="15">
       <c r="A592" s="122" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B592" s="122">
         <v>1</v>
@@ -22934,7 +22933,7 @@
         <v>497</v>
       </c>
       <c r="D592" s="122" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E592" s="123">
         <v>46336</v>
@@ -22946,15 +22945,15 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H592" s="122" t="s">
-        <v>488</v>
-      </c>
-      <c r="I592" s="158" t="s">
+        <v>490</v>
+      </c>
+      <c r="I592" s="156" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="593" spans="1:9" ht="15">
       <c r="A593" s="122" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B593" s="122">
         <v>1</v>
@@ -22963,7 +22962,7 @@
         <v>497</v>
       </c>
       <c r="D593" s="122" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E593" s="123">
         <v>46337</v>
@@ -22975,15 +22974,15 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H593" s="122" t="s">
-        <v>520</v>
-      </c>
-      <c r="I593" s="158" t="s">
+        <v>519</v>
+      </c>
+      <c r="I593" s="156" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="594" spans="1:9" ht="15">
       <c r="A594" s="122" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B594" s="122">
         <v>1</v>
@@ -22992,7 +22991,7 @@
         <v>497</v>
       </c>
       <c r="D594" s="122" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E594" s="123">
         <v>46338</v>
@@ -23004,15 +23003,15 @@
         <v>0.73958333333333337</v>
       </c>
       <c r="H594" s="122" t="s">
-        <v>506</v>
-      </c>
-      <c r="I594" s="159" t="s">
-        <v>517</v>
+        <v>505</v>
+      </c>
+      <c r="I594" s="157" t="s">
+        <v>516</v>
       </c>
     </row>
     <row r="595" spans="1:9" ht="15">
       <c r="A595" s="122" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B595" s="122">
         <v>1</v>
@@ -23021,7 +23020,7 @@
         <v>12</v>
       </c>
       <c r="D595" s="122" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="E595" s="123">
         <v>46339</v>
@@ -23033,15 +23032,15 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H595" s="122" t="s">
-        <v>434</v>
-      </c>
-      <c r="I595" s="158" t="s">
+        <v>435</v>
+      </c>
+      <c r="I595" s="156" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="596" spans="1:9" ht="15">
       <c r="A596" s="122" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B596" s="122">
         <v>1</v>
@@ -23050,7 +23049,7 @@
         <v>12</v>
       </c>
       <c r="D596" s="122" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="E596" s="123">
         <v>46339</v>
@@ -23062,15 +23061,15 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H596" s="122" t="s">
-        <v>434</v>
-      </c>
-      <c r="I596" s="159" t="s">
+        <v>435</v>
+      </c>
+      <c r="I596" s="157" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="597" spans="1:9" ht="15">
       <c r="A597" s="122" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B597" s="122">
         <v>1</v>
@@ -23079,7 +23078,7 @@
         <v>12</v>
       </c>
       <c r="D597" s="122" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="E597" s="123">
         <v>46339</v>
@@ -23091,15 +23090,15 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H597" s="122" t="s">
-        <v>434</v>
-      </c>
-      <c r="I597" s="158" t="s">
+        <v>435</v>
+      </c>
+      <c r="I597" s="156" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="598" spans="1:9" ht="15">
       <c r="A598" s="125" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B598" s="125">
         <v>1</v>
@@ -23108,7 +23107,7 @@
         <v>12</v>
       </c>
       <c r="D598" s="125" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="E598" s="126">
         <v>46339</v>
@@ -23120,15 +23119,15 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H598" s="125" t="s">
-        <v>434</v>
-      </c>
-      <c r="I598" s="159" t="s">
+        <v>435</v>
+      </c>
+      <c r="I598" s="157" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="599" spans="1:9" ht="15">
       <c r="A599" s="122" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B599" s="125">
         <v>1</v>
@@ -23149,15 +23148,15 @@
         <v>0.76041666666666663</v>
       </c>
       <c r="H599" s="122" t="s">
-        <v>374</v>
-      </c>
-      <c r="I599" s="159" t="s">
+        <v>375</v>
+      </c>
+      <c r="I599" s="157" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="600" spans="1:9" ht="15">
       <c r="A600" s="122" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B600" s="125">
         <v>1</v>
@@ -23180,22 +23179,22 @@
       <c r="H600" s="122" t="s">
         <v>355</v>
       </c>
-      <c r="I600" s="159" t="s">
+      <c r="I600" s="157" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="601" spans="1:9" ht="15">
       <c r="A601" s="122" t="s">
+        <v>525</v>
+      </c>
+      <c r="B601" s="125">
+        <v>1</v>
+      </c>
+      <c r="C601" s="125" t="s">
+        <v>12</v>
+      </c>
+      <c r="D601" s="122" t="s">
         <v>526</v>
-      </c>
-      <c r="B601" s="125">
-        <v>1</v>
-      </c>
-      <c r="C601" s="125" t="s">
-        <v>12</v>
-      </c>
-      <c r="D601" s="122" t="s">
-        <v>527</v>
       </c>
       <c r="E601" s="123">
         <v>46336</v>
@@ -23207,9 +23206,9 @@
         <v>0.76041666666666663</v>
       </c>
       <c r="H601" s="122" t="s">
-        <v>528</v>
-      </c>
-      <c r="I601" s="159" t="s">
+        <v>527</v>
+      </c>
+      <c r="I601" s="157" t="s">
         <v>53</v>
       </c>
     </row>
@@ -23257,175 +23256,175 @@
     <row r="1" spans="1:38" ht="20.100000000000001">
       <c r="A1" s="28"/>
       <c r="B1" s="29"/>
-      <c r="C1" s="155" t="s">
+      <c r="C1" s="163" t="s">
+        <v>528</v>
+      </c>
+      <c r="D1" s="164"/>
+      <c r="E1" s="164"/>
+      <c r="F1" s="164"/>
+      <c r="G1" s="164"/>
+      <c r="H1" s="164"/>
+      <c r="I1" s="163" t="s">
         <v>529</v>
       </c>
-      <c r="D1" s="156"/>
-      <c r="E1" s="156"/>
-      <c r="F1" s="156"/>
-      <c r="G1" s="156"/>
-      <c r="H1" s="156"/>
-      <c r="I1" s="155" t="s">
+      <c r="J1" s="164"/>
+      <c r="K1" s="164"/>
+      <c r="L1" s="164"/>
+      <c r="M1" s="164"/>
+      <c r="N1" s="164"/>
+      <c r="O1" s="164"/>
+      <c r="P1" s="164"/>
+      <c r="Q1" s="163" t="s">
         <v>530</v>
       </c>
-      <c r="J1" s="156"/>
-      <c r="K1" s="156"/>
-      <c r="L1" s="156"/>
-      <c r="M1" s="156"/>
-      <c r="N1" s="156"/>
-      <c r="O1" s="156"/>
-      <c r="P1" s="156"/>
-      <c r="Q1" s="155" t="s">
+      <c r="R1" s="164"/>
+      <c r="S1" s="164"/>
+      <c r="T1" s="164"/>
+      <c r="U1" s="164"/>
+      <c r="V1" s="164"/>
+      <c r="W1" s="164"/>
+      <c r="X1" s="163" t="s">
         <v>531</v>
       </c>
-      <c r="R1" s="156"/>
-      <c r="S1" s="156"/>
-      <c r="T1" s="156"/>
-      <c r="U1" s="156"/>
-      <c r="V1" s="156"/>
-      <c r="W1" s="156"/>
-      <c r="X1" s="155" t="s">
+      <c r="Y1" s="164"/>
+      <c r="Z1" s="164"/>
+      <c r="AA1" s="164"/>
+      <c r="AB1" s="164"/>
+      <c r="AC1" s="164"/>
+      <c r="AD1" s="164"/>
+      <c r="AE1" s="164"/>
+      <c r="AF1" s="163" t="s">
         <v>532</v>
       </c>
-      <c r="Y1" s="156"/>
-      <c r="Z1" s="156"/>
-      <c r="AA1" s="156"/>
-      <c r="AB1" s="156"/>
-      <c r="AC1" s="156"/>
-      <c r="AD1" s="156"/>
-      <c r="AE1" s="156"/>
-      <c r="AF1" s="155" t="s">
-        <v>533</v>
-      </c>
-      <c r="AG1" s="156"/>
-      <c r="AH1" s="156"/>
-      <c r="AI1" s="156"/>
-      <c r="AJ1" s="156"/>
+      <c r="AG1" s="164"/>
+      <c r="AH1" s="164"/>
+      <c r="AI1" s="164"/>
+      <c r="AJ1" s="164"/>
       <c r="AK1" s="30"/>
       <c r="AL1" s="30"/>
     </row>
     <row r="2" spans="1:38" ht="20.100000000000001">
       <c r="A2" s="31" t="s">
+        <v>533</v>
+      </c>
+      <c r="B2" s="32" t="s">
         <v>534</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="C2" s="33" t="s">
         <v>535</v>
       </c>
-      <c r="C2" s="33" t="s">
+      <c r="D2" s="34" t="s">
         <v>536</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="E2" s="34" t="s">
         <v>537</v>
       </c>
-      <c r="E2" s="34" t="s">
+      <c r="F2" s="34" t="s">
         <v>538</v>
       </c>
-      <c r="F2" s="34" t="s">
+      <c r="G2" s="34" t="s">
         <v>539</v>
       </c>
-      <c r="G2" s="34" t="s">
+      <c r="H2" s="35" t="s">
         <v>540</v>
       </c>
-      <c r="H2" s="35" t="s">
+      <c r="I2" s="33" t="s">
         <v>541</v>
       </c>
-      <c r="I2" s="33" t="s">
+      <c r="J2" s="33" t="s">
         <v>542</v>
       </c>
-      <c r="J2" s="33" t="s">
+      <c r="K2" s="33" t="s">
         <v>543</v>
       </c>
-      <c r="K2" s="33" t="s">
+      <c r="L2" s="34" t="s">
         <v>544</v>
       </c>
-      <c r="L2" s="34" t="s">
+      <c r="M2" s="34" t="s">
         <v>545</v>
       </c>
-      <c r="M2" s="34" t="s">
+      <c r="N2" s="34" t="s">
         <v>546</v>
       </c>
-      <c r="N2" s="34" t="s">
+      <c r="O2" s="34" t="s">
         <v>547</v>
       </c>
-      <c r="O2" s="34" t="s">
+      <c r="P2" s="34" t="s">
         <v>548</v>
       </c>
-      <c r="P2" s="34" t="s">
+      <c r="Q2" s="33" t="s">
+        <v>541</v>
+      </c>
+      <c r="R2" s="33" t="s">
+        <v>542</v>
+      </c>
+      <c r="S2" s="33" t="s">
+        <v>543</v>
+      </c>
+      <c r="T2" s="34" t="s">
+        <v>544</v>
+      </c>
+      <c r="U2" s="34" t="s">
+        <v>545</v>
+      </c>
+      <c r="V2" s="34" t="s">
+        <v>546</v>
+      </c>
+      <c r="W2" s="34" t="s">
+        <v>547</v>
+      </c>
+      <c r="X2" s="33" t="s">
+        <v>541</v>
+      </c>
+      <c r="Y2" s="33" t="s">
+        <v>542</v>
+      </c>
+      <c r="Z2" s="33" t="s">
+        <v>543</v>
+      </c>
+      <c r="AA2" s="34" t="s">
+        <v>544</v>
+      </c>
+      <c r="AB2" s="34" t="s">
+        <v>545</v>
+      </c>
+      <c r="AC2" s="34" t="s">
+        <v>546</v>
+      </c>
+      <c r="AD2" s="34" t="s">
+        <v>547</v>
+      </c>
+      <c r="AE2" s="35" t="s">
+        <v>548</v>
+      </c>
+      <c r="AF2" s="33" t="s">
+        <v>535</v>
+      </c>
+      <c r="AG2" s="34" t="s">
+        <v>536</v>
+      </c>
+      <c r="AH2" s="36" t="s">
+        <v>537</v>
+      </c>
+      <c r="AI2" s="34" t="s">
         <v>549</v>
       </c>
-      <c r="Q2" s="33" t="s">
-        <v>542</v>
-      </c>
-      <c r="R2" s="33" t="s">
-        <v>543</v>
-      </c>
-      <c r="S2" s="33" t="s">
-        <v>544</v>
-      </c>
-      <c r="T2" s="34" t="s">
-        <v>545</v>
-      </c>
-      <c r="U2" s="34" t="s">
-        <v>546</v>
-      </c>
-      <c r="V2" s="34" t="s">
-        <v>547</v>
-      </c>
-      <c r="W2" s="34" t="s">
-        <v>548</v>
-      </c>
-      <c r="X2" s="33" t="s">
-        <v>542</v>
-      </c>
-      <c r="Y2" s="33" t="s">
-        <v>543</v>
-      </c>
-      <c r="Z2" s="33" t="s">
-        <v>544</v>
-      </c>
-      <c r="AA2" s="34" t="s">
-        <v>545</v>
-      </c>
-      <c r="AB2" s="34" t="s">
-        <v>546</v>
-      </c>
-      <c r="AC2" s="34" t="s">
-        <v>547</v>
-      </c>
-      <c r="AD2" s="34" t="s">
-        <v>548</v>
-      </c>
-      <c r="AE2" s="35" t="s">
-        <v>549</v>
-      </c>
-      <c r="AF2" s="33" t="s">
-        <v>536</v>
-      </c>
-      <c r="AG2" s="34" t="s">
-        <v>537</v>
-      </c>
-      <c r="AH2" s="36" t="s">
-        <v>538</v>
-      </c>
-      <c r="AI2" s="34" t="s">
+      <c r="AJ2" s="35" t="s">
         <v>550</v>
       </c>
-      <c r="AJ2" s="35" t="s">
+      <c r="AK2" s="37" t="s">
         <v>551</v>
       </c>
-      <c r="AK2" s="37" t="s">
+      <c r="AL2" s="35" t="s">
         <v>552</v>
-      </c>
-      <c r="AL2" s="35" t="s">
-        <v>553</v>
       </c>
     </row>
     <row r="3" spans="1:38" ht="109.5" customHeight="1">
       <c r="A3" s="38" t="s">
+        <v>553</v>
+      </c>
+      <c r="B3" s="39" t="s">
         <v>554</v>
-      </c>
-      <c r="B3" s="39" t="s">
-        <v>555</v>
       </c>
       <c r="C3" s="40"/>
       <c r="D3" s="41"/>
@@ -23435,58 +23434,58 @@
       <c r="H3" s="43"/>
       <c r="I3" s="40"/>
       <c r="J3" s="44" t="s">
+        <v>555</v>
+      </c>
+      <c r="K3" s="45" t="s">
         <v>556</v>
       </c>
-      <c r="K3" s="45" t="s">
+      <c r="L3" s="45" t="s">
         <v>557</v>
       </c>
-      <c r="L3" s="45" t="s">
+      <c r="M3" s="45" t="s">
         <v>558</v>
       </c>
-      <c r="M3" s="45" t="s">
+      <c r="N3" s="45" t="s">
         <v>559</v>
       </c>
-      <c r="N3" s="45" t="s">
+      <c r="O3" s="45" t="s">
         <v>560</v>
       </c>
-      <c r="O3" s="45" t="s">
+      <c r="P3" s="46" t="s">
         <v>561</v>
       </c>
-      <c r="P3" s="46" t="s">
+      <c r="Q3" s="47" t="s">
         <v>562</v>
       </c>
-      <c r="Q3" s="47" t="s">
+      <c r="R3" s="48" t="s">
         <v>563</v>
       </c>
-      <c r="R3" s="48" t="s">
+      <c r="S3" s="48" t="s">
         <v>564</v>
       </c>
-      <c r="S3" s="48" t="s">
+      <c r="T3" s="48" t="s">
         <v>565</v>
-      </c>
-      <c r="T3" s="48" t="s">
-        <v>566</v>
       </c>
       <c r="U3" s="42"/>
       <c r="V3" s="42"/>
       <c r="W3" s="49"/>
       <c r="X3" s="50" t="s">
+        <v>566</v>
+      </c>
+      <c r="Y3" s="51" t="s">
         <v>567</v>
       </c>
-      <c r="Y3" s="51" t="s">
+      <c r="Z3" s="51" t="s">
         <v>568</v>
       </c>
-      <c r="Z3" s="51" t="s">
+      <c r="AA3" s="51" t="s">
         <v>569</v>
       </c>
-      <c r="AA3" s="51" t="s">
+      <c r="AB3" s="51" t="s">
         <v>570</v>
       </c>
-      <c r="AB3" s="51" t="s">
+      <c r="AC3" s="51" t="s">
         <v>571</v>
-      </c>
-      <c r="AC3" s="51" t="s">
-        <v>572</v>
       </c>
       <c r="AD3" s="49"/>
       <c r="AE3" s="52"/>
@@ -23500,7 +23499,7 @@
     </row>
     <row r="4" spans="1:38" ht="109.5" customHeight="1">
       <c r="A4" s="38" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B4" s="55">
         <v>30</v>
@@ -23513,58 +23512,58 @@
       <c r="H4" s="60"/>
       <c r="I4" s="56"/>
       <c r="J4" s="61" t="s">
+        <v>555</v>
+      </c>
+      <c r="K4" s="62" t="s">
         <v>556</v>
       </c>
-      <c r="K4" s="62" t="s">
+      <c r="L4" s="63" t="s">
         <v>557</v>
       </c>
-      <c r="L4" s="63" t="s">
+      <c r="M4" s="63" t="s">
         <v>558</v>
       </c>
-      <c r="M4" s="63" t="s">
+      <c r="N4" s="63" t="s">
         <v>559</v>
       </c>
-      <c r="N4" s="63" t="s">
+      <c r="O4" s="63" t="s">
         <v>560</v>
       </c>
-      <c r="O4" s="63" t="s">
+      <c r="P4" s="64" t="s">
         <v>561</v>
       </c>
-      <c r="P4" s="64" t="s">
+      <c r="Q4" s="65" t="s">
         <v>562</v>
       </c>
-      <c r="Q4" s="65" t="s">
+      <c r="R4" s="66" t="s">
         <v>563</v>
       </c>
-      <c r="R4" s="66" t="s">
+      <c r="S4" s="66" t="s">
         <v>564</v>
       </c>
-      <c r="S4" s="66" t="s">
+      <c r="T4" s="66" t="s">
         <v>565</v>
-      </c>
-      <c r="T4" s="66" t="s">
-        <v>566</v>
       </c>
       <c r="U4" s="58"/>
       <c r="V4" s="58"/>
       <c r="W4" s="67"/>
       <c r="X4" s="68" t="s">
+        <v>566</v>
+      </c>
+      <c r="Y4" s="69" t="s">
         <v>567</v>
       </c>
-      <c r="Y4" s="69" t="s">
+      <c r="Z4" s="69" t="s">
         <v>568</v>
       </c>
-      <c r="Z4" s="69" t="s">
+      <c r="AA4" s="69" t="s">
         <v>569</v>
       </c>
-      <c r="AA4" s="69" t="s">
+      <c r="AB4" s="69" t="s">
         <v>570</v>
       </c>
-      <c r="AB4" s="69" t="s">
+      <c r="AC4" s="69" t="s">
         <v>571</v>
-      </c>
-      <c r="AC4" s="69" t="s">
-        <v>572</v>
       </c>
       <c r="AD4" s="67"/>
       <c r="AE4" s="70"/>
@@ -23578,7 +23577,7 @@
     </row>
     <row r="5" spans="1:38" ht="109.5" customHeight="1">
       <c r="A5" s="38" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B5" s="55">
         <v>50</v>
@@ -23591,58 +23590,58 @@
       <c r="H5" s="60"/>
       <c r="I5" s="56"/>
       <c r="J5" s="61" t="s">
+        <v>555</v>
+      </c>
+      <c r="K5" s="62" t="s">
         <v>556</v>
       </c>
-      <c r="K5" s="62" t="s">
+      <c r="L5" s="63" t="s">
         <v>557</v>
       </c>
-      <c r="L5" s="63" t="s">
+      <c r="M5" s="63" t="s">
         <v>558</v>
       </c>
-      <c r="M5" s="63" t="s">
+      <c r="N5" s="63" t="s">
         <v>559</v>
       </c>
-      <c r="N5" s="63" t="s">
+      <c r="O5" s="63" t="s">
         <v>560</v>
       </c>
-      <c r="O5" s="63" t="s">
+      <c r="P5" s="64" t="s">
         <v>561</v>
       </c>
-      <c r="P5" s="64" t="s">
+      <c r="Q5" s="65" t="s">
         <v>562</v>
       </c>
-      <c r="Q5" s="65" t="s">
+      <c r="R5" s="76" t="s">
         <v>563</v>
       </c>
-      <c r="R5" s="76" t="s">
+      <c r="S5" s="76" t="s">
         <v>564</v>
       </c>
-      <c r="S5" s="76" t="s">
+      <c r="T5" s="76" t="s">
         <v>565</v>
-      </c>
-      <c r="T5" s="76" t="s">
-        <v>566</v>
       </c>
       <c r="U5" s="75"/>
       <c r="V5" s="75"/>
       <c r="W5" s="67"/>
       <c r="X5" s="68" t="s">
+        <v>566</v>
+      </c>
+      <c r="Y5" s="77" t="s">
         <v>567</v>
       </c>
-      <c r="Y5" s="77" t="s">
+      <c r="Z5" s="77" t="s">
         <v>568</v>
       </c>
-      <c r="Z5" s="77" t="s">
+      <c r="AA5" s="77" t="s">
         <v>569</v>
       </c>
-      <c r="AA5" s="77" t="s">
+      <c r="AB5" s="77" t="s">
         <v>570</v>
       </c>
-      <c r="AB5" s="77" t="s">
+      <c r="AC5" s="77" t="s">
         <v>571</v>
-      </c>
-      <c r="AC5" s="77" t="s">
-        <v>572</v>
       </c>
       <c r="AD5" s="67"/>
       <c r="AE5" s="70"/>
@@ -23656,7 +23655,7 @@
     </row>
     <row r="6" spans="1:38" ht="109.5" customHeight="1">
       <c r="A6" s="79" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="B6" s="55">
         <v>50</v>
@@ -23669,58 +23668,58 @@
       <c r="H6" s="82"/>
       <c r="I6" s="80"/>
       <c r="J6" s="61" t="s">
+        <v>555</v>
+      </c>
+      <c r="K6" s="62" t="s">
         <v>556</v>
       </c>
-      <c r="K6" s="62" t="s">
+      <c r="L6" s="63" t="s">
         <v>557</v>
       </c>
-      <c r="L6" s="63" t="s">
+      <c r="M6" s="63" t="s">
         <v>558</v>
       </c>
-      <c r="M6" s="63" t="s">
+      <c r="N6" s="63" t="s">
         <v>559</v>
       </c>
-      <c r="N6" s="63" t="s">
+      <c r="O6" s="63" t="s">
         <v>560</v>
       </c>
-      <c r="O6" s="63" t="s">
+      <c r="P6" s="64" t="s">
         <v>561</v>
       </c>
-      <c r="P6" s="64" t="s">
+      <c r="Q6" s="83" t="s">
         <v>562</v>
       </c>
-      <c r="Q6" s="83" t="s">
+      <c r="R6" s="76" t="s">
         <v>563</v>
       </c>
-      <c r="R6" s="76" t="s">
+      <c r="S6" s="76" t="s">
         <v>564</v>
       </c>
-      <c r="S6" s="76" t="s">
+      <c r="T6" s="76" t="s">
         <v>565</v>
-      </c>
-      <c r="T6" s="76" t="s">
-        <v>566</v>
       </c>
       <c r="U6" s="75"/>
       <c r="V6" s="75"/>
       <c r="W6" s="84"/>
       <c r="X6" s="85" t="s">
+        <v>566</v>
+      </c>
+      <c r="Y6" s="77" t="s">
         <v>567</v>
       </c>
-      <c r="Y6" s="77" t="s">
+      <c r="Z6" s="77" t="s">
         <v>568</v>
       </c>
-      <c r="Z6" s="77" t="s">
+      <c r="AA6" s="77" t="s">
         <v>569</v>
       </c>
-      <c r="AA6" s="77" t="s">
+      <c r="AB6" s="77" t="s">
         <v>570</v>
       </c>
-      <c r="AB6" s="77" t="s">
+      <c r="AC6" s="77" t="s">
         <v>571</v>
-      </c>
-      <c r="AC6" s="77" t="s">
-        <v>572</v>
       </c>
       <c r="AD6" s="84"/>
       <c r="AE6" s="70"/>
@@ -23734,7 +23733,7 @@
     </row>
     <row r="7" spans="1:38" ht="109.5" customHeight="1">
       <c r="A7" s="79" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="B7" s="55">
         <v>50</v>
@@ -23747,58 +23746,58 @@
       <c r="H7" s="82"/>
       <c r="I7" s="80"/>
       <c r="J7" s="61" t="s">
+        <v>555</v>
+      </c>
+      <c r="K7" s="62" t="s">
         <v>556</v>
       </c>
-      <c r="K7" s="62" t="s">
+      <c r="L7" s="63" t="s">
         <v>557</v>
       </c>
-      <c r="L7" s="63" t="s">
+      <c r="M7" s="63" t="s">
         <v>558</v>
       </c>
-      <c r="M7" s="63" t="s">
+      <c r="N7" s="63" t="s">
         <v>559</v>
       </c>
-      <c r="N7" s="63" t="s">
+      <c r="O7" s="63" t="s">
         <v>560</v>
       </c>
-      <c r="O7" s="63" t="s">
+      <c r="P7" s="64" t="s">
         <v>561</v>
       </c>
-      <c r="P7" s="64" t="s">
+      <c r="Q7" s="83" t="s">
         <v>562</v>
       </c>
-      <c r="Q7" s="83" t="s">
+      <c r="R7" s="76" t="s">
         <v>563</v>
       </c>
-      <c r="R7" s="76" t="s">
+      <c r="S7" s="76" t="s">
         <v>564</v>
       </c>
-      <c r="S7" s="76" t="s">
+      <c r="T7" s="76" t="s">
         <v>565</v>
-      </c>
-      <c r="T7" s="76" t="s">
-        <v>566</v>
       </c>
       <c r="U7" s="75"/>
       <c r="V7" s="75"/>
       <c r="W7" s="84"/>
       <c r="X7" s="85" t="s">
+        <v>566</v>
+      </c>
+      <c r="Y7" s="77" t="s">
         <v>567</v>
       </c>
-      <c r="Y7" s="77" t="s">
+      <c r="Z7" s="77" t="s">
         <v>568</v>
       </c>
-      <c r="Z7" s="77" t="s">
+      <c r="AA7" s="77" t="s">
         <v>569</v>
       </c>
-      <c r="AA7" s="77" t="s">
+      <c r="AB7" s="77" t="s">
         <v>570</v>
       </c>
-      <c r="AB7" s="77" t="s">
+      <c r="AC7" s="77" t="s">
         <v>571</v>
-      </c>
-      <c r="AC7" s="77" t="s">
-        <v>572</v>
       </c>
       <c r="AD7" s="84"/>
       <c r="AE7" s="70"/>
@@ -23812,7 +23811,7 @@
     </row>
     <row r="8" spans="1:38" ht="109.5" customHeight="1">
       <c r="A8" s="79" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B8" s="55">
         <v>48</v>
@@ -23825,58 +23824,58 @@
       <c r="H8" s="82"/>
       <c r="I8" s="80"/>
       <c r="J8" s="61" t="s">
+        <v>555</v>
+      </c>
+      <c r="K8" s="62" t="s">
         <v>556</v>
       </c>
-      <c r="K8" s="62" t="s">
+      <c r="L8" s="63" t="s">
         <v>557</v>
       </c>
-      <c r="L8" s="63" t="s">
+      <c r="M8" s="63" t="s">
         <v>558</v>
       </c>
-      <c r="M8" s="63" t="s">
+      <c r="N8" s="63" t="s">
         <v>559</v>
       </c>
-      <c r="N8" s="63" t="s">
+      <c r="O8" s="63" t="s">
         <v>560</v>
       </c>
-      <c r="O8" s="63" t="s">
+      <c r="P8" s="64" t="s">
         <v>561</v>
       </c>
-      <c r="P8" s="64" t="s">
+      <c r="Q8" s="83" t="s">
         <v>562</v>
       </c>
-      <c r="Q8" s="83" t="s">
+      <c r="R8" s="76" t="s">
         <v>563</v>
       </c>
-      <c r="R8" s="76" t="s">
+      <c r="S8" s="76" t="s">
         <v>564</v>
       </c>
-      <c r="S8" s="76" t="s">
+      <c r="T8" s="76" t="s">
         <v>565</v>
-      </c>
-      <c r="T8" s="76" t="s">
-        <v>566</v>
       </c>
       <c r="U8" s="75"/>
       <c r="V8" s="75"/>
       <c r="W8" s="84"/>
       <c r="X8" s="85" t="s">
+        <v>566</v>
+      </c>
+      <c r="Y8" s="77" t="s">
         <v>567</v>
       </c>
-      <c r="Y8" s="77" t="s">
+      <c r="Z8" s="77" t="s">
         <v>568</v>
       </c>
-      <c r="Z8" s="77" t="s">
+      <c r="AA8" s="77" t="s">
         <v>569</v>
       </c>
-      <c r="AA8" s="77" t="s">
+      <c r="AB8" s="77" t="s">
         <v>570</v>
       </c>
-      <c r="AB8" s="77" t="s">
+      <c r="AC8" s="77" t="s">
         <v>571</v>
-      </c>
-      <c r="AC8" s="77" t="s">
-        <v>572</v>
       </c>
       <c r="AD8" s="84"/>
       <c r="AE8" s="70"/>
@@ -23890,7 +23889,7 @@
     </row>
     <row r="9" spans="1:38" ht="109.5" customHeight="1">
       <c r="A9" s="90" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B9" s="91">
         <v>40</v>
@@ -23898,65 +23897,65 @@
       <c r="C9" s="92"/>
       <c r="D9" s="93"/>
       <c r="E9" s="94" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="F9" s="95"/>
       <c r="G9" s="95"/>
       <c r="H9" s="96"/>
       <c r="I9" s="92"/>
       <c r="J9" s="97" t="s">
+        <v>555</v>
+      </c>
+      <c r="K9" s="98" t="s">
         <v>556</v>
       </c>
-      <c r="K9" s="98" t="s">
+      <c r="L9" s="99" t="s">
         <v>557</v>
       </c>
-      <c r="L9" s="99" t="s">
+      <c r="M9" s="99" t="s">
         <v>558</v>
       </c>
-      <c r="M9" s="99" t="s">
+      <c r="N9" s="99" t="s">
         <v>559</v>
       </c>
-      <c r="N9" s="99" t="s">
+      <c r="O9" s="99" t="s">
         <v>560</v>
       </c>
-      <c r="O9" s="99" t="s">
+      <c r="P9" s="100" t="s">
         <v>561</v>
       </c>
-      <c r="P9" s="100" t="s">
+      <c r="Q9" s="101" t="s">
         <v>562</v>
       </c>
-      <c r="Q9" s="101" t="s">
+      <c r="R9" s="102" t="s">
         <v>563</v>
       </c>
-      <c r="R9" s="102" t="s">
+      <c r="S9" s="102" t="s">
         <v>564</v>
       </c>
-      <c r="S9" s="102" t="s">
+      <c r="T9" s="102" t="s">
         <v>565</v>
-      </c>
-      <c r="T9" s="102" t="s">
-        <v>566</v>
       </c>
       <c r="U9" s="103"/>
       <c r="V9" s="103"/>
       <c r="W9" s="104"/>
       <c r="X9" s="105" t="s">
+        <v>566</v>
+      </c>
+      <c r="Y9" s="106" t="s">
         <v>567</v>
       </c>
-      <c r="Y9" s="106" t="s">
-        <v>568</v>
-      </c>
       <c r="Z9" s="106" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA9" s="106" t="s">
+        <v>569</v>
+      </c>
+      <c r="AB9" s="106" t="s">
         <v>570</v>
       </c>
-      <c r="AB9" s="106" t="s">
+      <c r="AC9" s="106" t="s">
         <v>571</v>
-      </c>
-      <c r="AC9" s="106" t="s">
-        <v>572</v>
       </c>
       <c r="AD9" s="104"/>
       <c r="AE9" s="107"/>

</xml_diff>